<commit_message>
Simulation tab: add Session E conclusions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tKeYTtjF85cuvm1dpYiVi
</commit_message>
<xml_diff>
--- a/model/GRG_model_v0.6.xlsx
+++ b/model/GRG_model_v0.6.xlsx
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="595">
   <si>
     <t xml:space="preserve">Greggs three-statement forecast model – Notes</t>
   </si>
@@ -1992,6 +1992,15 @@
   </si>
   <si>
     <t xml:space="preserve">Your conclusions (Session E, in your own words)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In 90% of 10,000 runs FY26 underlying profit beats FY25's £172m, with a likely range of £170–190m, so I am confident profit grows.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash stays positive in every run and falls below £50m in only 1%: with capex falling, Greggs can fund openings, restructuring and dividends without new debt, after negative free cash flow in FY25.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I would watch like-for-like growth: margin moves profit most (£53m), but LFL moves it £23m directly, pulls margin with it through operating leverage, and is the trend that has slowed from 18% to 2%.</t>
   </si>
   <si>
     <t xml:space="preserve">Checks – every row should show 0 (green). Red means something does not tie.</t>
@@ -2377,7 +2386,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="88">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2706,36 +2715,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2845,9 +2838,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>592200</xdr:colOff>
+      <xdr:colOff>591840</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>122400</xdr:rowOff>
+      <xdr:rowOff>122040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2860,8 +2853,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11466360" y="571680"/>
-          <a:ext cx="6095520" cy="3200040"/>
+          <a:off x="11466360" y="570600"/>
+          <a:ext cx="6095160" cy="3199680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2882,9 +2875,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>592200</xdr:colOff>
+      <xdr:colOff>591840</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2897,8 +2890,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11466360" y="4191120"/>
-          <a:ext cx="6095520" cy="2895120"/>
+          <a:off x="11466360" y="4190040"/>
+          <a:ext cx="6095160" cy="2894760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3660,20 +3653,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="35" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C4" s="35" t="s">
         <v>85</v>
@@ -3702,404 +3695,404 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="90" t="n">
+      <c r="C5" s="86" t="n">
         <f aca="false">ROUND(Historical!C13-Historical!C30,1)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="90" t="n">
+      <c r="D5" s="86" t="n">
         <f aca="false">ROUND(Historical!D13-Historical!D30,1)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="90" t="n">
+      <c r="E5" s="86" t="n">
         <f aca="false">ROUND(Historical!E13-Historical!E30,1)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="90" t="n">
+      <c r="F5" s="86" t="n">
         <f aca="false">ROUND(Historical!F13-Historical!F30,1)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="90" t="n">
+      <c r="G5" s="86" t="n">
         <f aca="false">ROUND(Historical!G13-Historical!G30,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B6" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="90" t="n">
+      <c r="C6" s="86" t="n">
         <f aca="false">ROUND(Historical!C16-Historical!C31,1)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="90" t="n">
+      <c r="D6" s="86" t="n">
         <f aca="false">ROUND(Historical!D16-Historical!D31,1)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="90" t="n">
+      <c r="E6" s="86" t="n">
         <f aca="false">ROUND(Historical!E16-Historical!E31,1)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="90" t="n">
+      <c r="F6" s="86" t="n">
         <f aca="false">ROUND(Historical!F16-Historical!F31,1)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="90" t="n">
+      <c r="G6" s="86" t="n">
         <f aca="false">ROUND(Historical!G16-Historical!G31,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="90" t="n">
+      <c r="C7" s="86" t="n">
         <f aca="false">ROUND(Historical!C18-Historical!C32,1)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="90" t="n">
+      <c r="D7" s="86" t="n">
         <f aca="false">ROUND(Historical!D18-Historical!D32,1)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="90" t="n">
+      <c r="E7" s="86" t="n">
         <f aca="false">ROUND(Historical!E18-Historical!E32,1)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="90" t="n">
+      <c r="F7" s="86" t="n">
         <f aca="false">ROUND(Historical!F18-Historical!F32,1)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="90" t="n">
+      <c r="G7" s="86" t="n">
         <f aca="false">ROUND(Historical!G18-Historical!G32,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="90" t="n">
+      <c r="C8" s="86" t="n">
         <f aca="false">ROUND(Historical!C25-Historical!C33,1)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="90" t="n">
+      <c r="D8" s="86" t="n">
         <f aca="false">ROUND(Historical!D25-Historical!D33,1)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="90" t="n">
+      <c r="E8" s="86" t="n">
         <f aca="false">ROUND(Historical!E25-Historical!E33,1)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="90" t="n">
+      <c r="F8" s="86" t="n">
         <f aca="false">ROUND(Historical!F25-Historical!F33,1)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="90" t="n">
+      <c r="G8" s="86" t="n">
         <f aca="false">ROUND(Historical!G25-Historical!G33,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="24" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="90" t="n">
+      <c r="C9" s="86" t="n">
         <f aca="false">ROUND(Historical!C36+Historical!C37-Historical!C7,1)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="90" t="n">
+      <c r="D9" s="86" t="n">
         <f aca="false">ROUND(Historical!D36+Historical!D37-Historical!D7,1)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="90" t="n">
+      <c r="E9" s="86" t="n">
         <f aca="false">ROUND(Historical!E36+Historical!E37-Historical!E7,1)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="90" t="n">
+      <c r="F9" s="86" t="n">
         <f aca="false">ROUND(Historical!F36+Historical!F37-Historical!F7,1)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="90" t="n">
+      <c r="G9" s="86" t="n">
         <f aca="false">ROUND(Historical!G36+Historical!G37-Historical!G7,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="90" t="n">
+      <c r="C10" s="86" t="n">
         <f aca="false">ROUND(Historical!C63-Historical!C83,1)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="90" t="n">
+      <c r="D10" s="86" t="n">
         <f aca="false">ROUND(Historical!D63-Historical!D83,1)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="90" t="n">
+      <c r="E10" s="86" t="n">
         <f aca="false">ROUND(Historical!E63-Historical!E83,1)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="90" t="n">
+      <c r="F10" s="86" t="n">
         <f aca="false">ROUND(Historical!F63-Historical!F83,1)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="90" t="n">
+      <c r="G10" s="86" t="n">
         <f aca="false">ROUND(Historical!G63-Historical!G83,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B11" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="90" t="n">
+      <c r="C11" s="86" t="n">
         <f aca="false">ROUND(Historical!C77-Historical!C84,1)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="90" t="n">
+      <c r="D11" s="86" t="n">
         <f aca="false">ROUND(Historical!D77-Historical!D84,1)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="90" t="n">
+      <c r="E11" s="86" t="n">
         <f aca="false">ROUND(Historical!E77-Historical!E84,1)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="90" t="n">
+      <c r="F11" s="86" t="n">
         <f aca="false">ROUND(Historical!F77-Historical!F84,1)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="90" t="n">
+      <c r="G11" s="86" t="n">
         <f aca="false">ROUND(Historical!G77-Historical!G84,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>560</v>
-      </c>
-      <c r="C12" s="90" t="n">
+        <v>563</v>
+      </c>
+      <c r="C12" s="86" t="n">
         <f aca="false">ROUND(Historical!C77-Historical!C82,1)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="90" t="n">
+      <c r="D12" s="86" t="n">
         <f aca="false">ROUND(Historical!D77-Historical!D82,1)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="90" t="n">
+      <c r="E12" s="86" t="n">
         <f aca="false">ROUND(Historical!E77-Historical!E82,1)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="90" t="n">
+      <c r="F12" s="86" t="n">
         <f aca="false">ROUND(Historical!F77-Historical!F82,1)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="90" t="n">
+      <c r="G12" s="86" t="n">
         <f aca="false">ROUND(Historical!G77-Historical!G82,1)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="90" t="n">
+      <c r="H12" s="86" t="n">
         <f aca="false">ROUND(Forecast!H77-Forecast!H82,1)</f>
         <v>0</v>
       </c>
-      <c r="I12" s="90" t="n">
+      <c r="I12" s="86" t="n">
         <f aca="false">ROUND(Forecast!I77-Forecast!I82,1)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="90" t="n">
+      <c r="J12" s="86" t="n">
         <f aca="false">ROUND(Forecast!J77-Forecast!J82,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="24" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>560</v>
-      </c>
-      <c r="C13" s="90" t="n">
+        <v>563</v>
+      </c>
+      <c r="C13" s="86" t="n">
         <f aca="false">ROUND(Historical!C113-Historical!C61,1)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="90" t="n">
+      <c r="D13" s="86" t="n">
         <f aca="false">ROUND(Historical!D113-Historical!D61,1)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="90" t="n">
+      <c r="E13" s="86" t="n">
         <f aca="false">ROUND(Historical!E113-Historical!E61,1)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="90" t="n">
+      <c r="F13" s="86" t="n">
         <f aca="false">ROUND(Historical!F113-Historical!F61,1)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="90" t="n">
+      <c r="G13" s="86" t="n">
         <f aca="false">ROUND(Historical!G113-Historical!G61,1)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="90" t="n">
+      <c r="H13" s="86" t="n">
         <f aca="false">ROUND(Forecast!H113-Forecast!H61,1)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="90" t="n">
+      <c r="I13" s="86" t="n">
         <f aca="false">ROUND(Forecast!I113-Forecast!I61,1)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="90" t="n">
+      <c r="J13" s="86" t="n">
         <f aca="false">ROUND(Forecast!J113-Forecast!J61,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="24" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="90" t="n">
+      <c r="C14" s="86" t="n">
         <f aca="false">ROUND(Historical!C111-Historical!C114,1)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="90" t="n">
+      <c r="D14" s="86" t="n">
         <f aca="false">ROUND(Historical!D111-Historical!D114,1)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="90" t="n">
+      <c r="E14" s="86" t="n">
         <f aca="false">ROUND(Historical!E111-Historical!E114,1)</f>
         <v>-0</v>
       </c>
-      <c r="F14" s="90" t="n">
+      <c r="F14" s="86" t="n">
         <f aca="false">ROUND(Historical!F111-Historical!F114,1)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="90" t="n">
+      <c r="G14" s="86" t="n">
         <f aca="false">ROUND(Historical!G111-Historical!G114,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="90" t="n">
+      <c r="C15" s="86" t="n">
         <f aca="false">ROUND(Historical!C138-Historical!C92,1)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="90" t="n">
+      <c r="D15" s="86" t="n">
         <f aca="false">ROUND(Historical!D138-Historical!D92,1)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="90" t="n">
+      <c r="E15" s="86" t="n">
         <f aca="false">ROUND(Historical!E138-Historical!E92,1)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="90" t="n">
+      <c r="F15" s="86" t="n">
         <f aca="false">ROUND(Historical!F138-Historical!F92,1)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="90" t="n">
+      <c r="G15" s="86" t="n">
         <f aca="false">ROUND(Historical!G138-Historical!G92,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="90" t="n">
+      <c r="C16" s="86" t="n">
         <f aca="false">ROUND(Historical!C121-Historical!C18,1)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="90" t="n">
+      <c r="D16" s="86" t="n">
         <f aca="false">ROUND(Historical!D121-Historical!D18,1)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="90" t="n">
+      <c r="E16" s="86" t="n">
         <f aca="false">ROUND(Historical!E121-Historical!E18,1)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="90" t="n">
+      <c r="F16" s="86" t="n">
         <f aca="false">ROUND(Historical!F121-Historical!F18,1)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="90" t="n">
+      <c r="G16" s="86" t="n">
         <f aca="false">ROUND(Historical!G121-Historical!G18,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="24" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="90" t="n">
+      <c r="C17" s="86" t="n">
         <f aca="false">ROUND(Historical!C46,1)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="90" t="n">
+      <c r="D17" s="86" t="n">
         <f aca="false">ROUND(Historical!D46,1)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="90" t="n">
+      <c r="E17" s="86" t="n">
         <f aca="false">ROUND(Historical!E46,1)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="90" t="n">
+      <c r="F17" s="86" t="n">
         <f aca="false">ROUND(Historical!F46,1)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="90" t="n">
+      <c r="G17" s="86" t="n">
         <f aca="false">ROUND(Historical!G46,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="44" t="s">
-        <v>566</v>
-      </c>
-      <c r="C19" s="91" t="n">
+        <v>569</v>
+      </c>
+      <c r="C19" s="87" t="n">
         <f aca="false">SUMPRODUCT(ABS(C5:G17))</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="44" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C20" s="26" t="str">
         <f aca="false">IF(C19&lt;0.05,"OK","CHECK")</f>
@@ -4108,145 +4101,145 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="44" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="24" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="90" t="n">
+      <c r="C23" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!C9:C13)=0,"",IF(ABS('Tax &amp; Audit'!C16)&lt;0.15,0,ROUND('Tax &amp; Audit'!C16,1)))</f>
         <v>0</v>
       </c>
-      <c r="D23" s="90" t="n">
+      <c r="D23" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!D9:D13)=0,"",IF(ABS('Tax &amp; Audit'!D16)&lt;0.15,0,ROUND('Tax &amp; Audit'!D16,1)))</f>
         <v>0</v>
       </c>
-      <c r="E23" s="90" t="n">
+      <c r="E23" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!E9:E13)=0,"",IF(ABS('Tax &amp; Audit'!E16)&lt;0.15,0,ROUND('Tax &amp; Audit'!E16,1)))</f>
         <v>0</v>
       </c>
-      <c r="F23" s="90" t="n">
+      <c r="F23" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!F9:F13)=0,"",IF(ABS('Tax &amp; Audit'!F16)&lt;0.15,0,ROUND('Tax &amp; Audit'!F16,1)))</f>
         <v>0</v>
       </c>
-      <c r="G23" s="90" t="n">
+      <c r="G23" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!G9:G13)=0,"",IF(ABS('Tax &amp; Audit'!G16)&lt;0.15,0,ROUND('Tax &amp; Audit'!G16,1)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="24" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="90" t="n">
+      <c r="C24" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!C22:C23)=0,"",ROUND('Tax &amp; Audit'!C25,1))</f>
         <v>0</v>
       </c>
-      <c r="D24" s="90" t="n">
+      <c r="D24" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!D22:D23)=0,"",ROUND('Tax &amp; Audit'!D25,1))</f>
         <v>0</v>
       </c>
-      <c r="E24" s="90" t="n">
+      <c r="E24" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!E22:E23)=0,"",ROUND('Tax &amp; Audit'!E25,1))</f>
         <v>0</v>
       </c>
-      <c r="F24" s="90" t="n">
+      <c r="F24" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!F22:F23)=0,"",ROUND('Tax &amp; Audit'!F25,1))</f>
         <v>0</v>
       </c>
-      <c r="G24" s="90" t="n">
+      <c r="G24" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!G22:G23)=0,"",ROUND('Tax &amp; Audit'!G25,1))</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="24" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="90" t="n">
+      <c r="C25" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!C31:C33)=0,"",ROUND('Tax &amp; Audit'!C36,1))</f>
         <v>0</v>
       </c>
-      <c r="D25" s="90" t="n">
+      <c r="D25" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!D31:D33)=0,"",ROUND('Tax &amp; Audit'!D36,1))</f>
         <v>0</v>
       </c>
-      <c r="E25" s="90" t="n">
+      <c r="E25" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!E31:E33)=0,"",ROUND('Tax &amp; Audit'!E36,1))</f>
         <v>0</v>
       </c>
-      <c r="F25" s="90" t="n">
+      <c r="F25" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!F31:F33)=0,"",ROUND('Tax &amp; Audit'!F36,1))</f>
         <v>0</v>
       </c>
-      <c r="G25" s="90" t="n">
+      <c r="G25" s="86" t="n">
         <f aca="false">IF(COUNT('Tax &amp; Audit'!G31:G33)=0,"",ROUND('Tax &amp; Audit'!G36,1))</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="44" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="35" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C29" s="35" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D29" s="35" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B30" s="67"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B31" s="67"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B32" s="67"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B33" s="67"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B34" s="67"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B35" s="67"/>
     </row>
@@ -4299,47 +4292,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="44" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="44" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="44" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="44" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="44" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="44" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="44" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="44" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
     </row>
   </sheetData>
@@ -15668,691 +15661,723 @@
   <dimension ref="A1:I42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="82" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="83" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="54" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="84" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="59" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="85" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="58" t="s">
         <v>523</v>
       </c>
-      <c r="B5" s="85" t="s">
+      <c r="B5" s="58" t="s">
         <v>423</v>
       </c>
-      <c r="C5" s="85" t="s">
+      <c r="C5" s="58" t="s">
         <v>524</v>
       </c>
-      <c r="D5" s="85" t="s">
+      <c r="D5" s="58" t="s">
         <v>525</v>
       </c>
-      <c r="E5" s="85" t="s">
+      <c r="E5" s="58" t="s">
         <v>526</v>
       </c>
-      <c r="F5" s="85" t="s">
+      <c r="F5" s="58" t="s">
         <v>527</v>
       </c>
-      <c r="G5" s="85" t="s">
+      <c r="G5" s="58" t="s">
         <v>528</v>
       </c>
-      <c r="H5" s="85" t="s">
+      <c r="H5" s="58" t="s">
         <v>529</v>
       </c>
-      <c r="I5" s="85" t="s">
+      <c r="I5" s="58" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="86" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="86" t="s">
+      <c r="B6" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="87" t="n">
+      <c r="C6" s="83" t="n">
         <v>2262.2</v>
       </c>
-      <c r="D6" s="87" t="n">
+      <c r="D6" s="83" t="n">
         <v>2272.5</v>
       </c>
-      <c r="E6" s="87" t="n">
+      <c r="E6" s="83" t="n">
         <v>2280.2</v>
       </c>
-      <c r="F6" s="87" t="n">
+      <c r="F6" s="83" t="n">
         <v>2287.7</v>
       </c>
-      <c r="G6" s="87" t="n">
+      <c r="G6" s="83" t="n">
         <v>2297.7</v>
       </c>
-      <c r="H6" s="87" t="n">
+      <c r="H6" s="83" t="n">
         <v>2280.1</v>
       </c>
-      <c r="I6" s="87" t="n">
+      <c r="I6" s="83" t="n">
         <v>2283.6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="86" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="86" t="s">
+      <c r="B7" s="63" t="s">
         <v>238</v>
       </c>
-      <c r="C7" s="87" t="n">
+      <c r="C7" s="83" t="n">
         <v>2357.2</v>
       </c>
-      <c r="D7" s="87" t="n">
+      <c r="D7" s="83" t="n">
         <v>2389.1</v>
       </c>
-      <c r="E7" s="87" t="n">
+      <c r="E7" s="83" t="n">
         <v>2412.6</v>
       </c>
-      <c r="F7" s="87" t="n">
+      <c r="F7" s="83" t="n">
         <v>2435.1</v>
       </c>
-      <c r="G7" s="87" t="n">
+      <c r="G7" s="83" t="n">
         <v>2466</v>
       </c>
-      <c r="H7" s="87" t="n">
+      <c r="H7" s="83" t="n">
         <v>2412</v>
       </c>
-      <c r="I7" s="87" t="n">
+      <c r="I7" s="83" t="n">
         <v>2421.1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="86" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="86" t="s">
+      <c r="B8" s="63" t="s">
         <v>239</v>
       </c>
-      <c r="C8" s="87" t="n">
+      <c r="C8" s="83" t="n">
         <v>2456.4</v>
       </c>
-      <c r="D8" s="87" t="n">
+      <c r="D8" s="83" t="n">
         <v>2512.3</v>
       </c>
-      <c r="E8" s="87" t="n">
+      <c r="E8" s="83" t="n">
         <v>2553.6</v>
       </c>
-      <c r="F8" s="87" t="n">
+      <c r="F8" s="83" t="n">
         <v>2593.4</v>
       </c>
-      <c r="G8" s="87" t="n">
+      <c r="G8" s="83" t="n">
         <v>2648.8</v>
       </c>
-      <c r="H8" s="87" t="n">
+      <c r="H8" s="83" t="n">
         <v>2553</v>
       </c>
-      <c r="I8" s="87" t="n">
+      <c r="I8" s="83" t="n">
         <v>2566.8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="86" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="B9" s="86" t="s">
+      <c r="B9" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="87" t="n">
+      <c r="C9" s="83" t="n">
         <v>169.8</v>
       </c>
-      <c r="D9" s="87" t="n">
+      <c r="D9" s="83" t="n">
         <v>175.6</v>
       </c>
-      <c r="E9" s="87" t="n">
+      <c r="E9" s="83" t="n">
         <v>179.9</v>
       </c>
-      <c r="F9" s="87" t="n">
+      <c r="F9" s="83" t="n">
         <v>184.1</v>
       </c>
-      <c r="G9" s="87" t="n">
+      <c r="G9" s="83" t="n">
         <v>189.9</v>
       </c>
-      <c r="H9" s="87" t="n">
+      <c r="H9" s="83" t="n">
         <v>179.9</v>
       </c>
-      <c r="I9" s="87" t="n">
+      <c r="I9" s="83" t="n">
         <v>180.2</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="86" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="63" t="s">
         <v>238</v>
       </c>
-      <c r="C10" s="87" t="n">
+      <c r="C10" s="83" t="n">
         <v>176.8</v>
       </c>
-      <c r="D10" s="87" t="n">
+      <c r="D10" s="83" t="n">
         <v>187.9</v>
       </c>
-      <c r="E10" s="87" t="n">
+      <c r="E10" s="83" t="n">
         <v>196</v>
       </c>
-      <c r="F10" s="87" t="n">
+      <c r="F10" s="83" t="n">
         <v>204.2</v>
       </c>
-      <c r="G10" s="87" t="n">
+      <c r="G10" s="83" t="n">
         <v>215.3</v>
       </c>
-      <c r="H10" s="87" t="n">
+      <c r="H10" s="83" t="n">
         <v>196.1</v>
       </c>
-      <c r="I10" s="87" t="n">
+      <c r="I10" s="83" t="n">
         <v>196.9</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="86" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="B11" s="86" t="s">
+      <c r="B11" s="63" t="s">
         <v>239</v>
       </c>
-      <c r="C11" s="87" t="n">
+      <c r="C11" s="83" t="n">
         <v>193</v>
       </c>
-      <c r="D11" s="87" t="n">
+      <c r="D11" s="83" t="n">
         <v>206.2</v>
       </c>
-      <c r="E11" s="87" t="n">
+      <c r="E11" s="83" t="n">
         <v>216.1</v>
       </c>
-      <c r="F11" s="87" t="n">
+      <c r="F11" s="83" t="n">
         <v>226</v>
       </c>
-      <c r="G11" s="87" t="n">
+      <c r="G11" s="83" t="n">
         <v>239.6</v>
       </c>
-      <c r="H11" s="87" t="n">
+      <c r="H11" s="83" t="n">
         <v>216.2</v>
       </c>
-      <c r="I11" s="87" t="n">
+      <c r="I11" s="83" t="n">
         <v>217.6</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="86" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="63" t="s">
         <v>215</v>
       </c>
-      <c r="B12" s="86" t="s">
+      <c r="B12" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="C12" s="87" t="n">
+      <c r="C12" s="83" t="n">
         <v>71.3</v>
       </c>
-      <c r="D12" s="87" t="n">
+      <c r="D12" s="83" t="n">
         <v>77.8</v>
       </c>
-      <c r="E12" s="87" t="n">
+      <c r="E12" s="83" t="n">
         <v>82.4</v>
       </c>
-      <c r="F12" s="87" t="n">
+      <c r="F12" s="83" t="n">
         <v>86.9</v>
       </c>
-      <c r="G12" s="87" t="n">
+      <c r="G12" s="83" t="n">
         <v>93</v>
       </c>
-      <c r="H12" s="87" t="n">
+      <c r="H12" s="83" t="n">
         <v>82.3</v>
       </c>
-      <c r="I12" s="87" t="n">
+      <c r="I12" s="83" t="n">
         <v>84.6</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="86" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="63" t="s">
         <v>215</v>
       </c>
-      <c r="B13" s="86" t="s">
+      <c r="B13" s="63" t="s">
         <v>238</v>
       </c>
-      <c r="C13" s="87" t="n">
+      <c r="C13" s="83" t="n">
         <v>62.8</v>
       </c>
-      <c r="D13" s="87" t="n">
+      <c r="D13" s="83" t="n">
         <v>77.1</v>
       </c>
-      <c r="E13" s="87" t="n">
+      <c r="E13" s="83" t="n">
         <v>87.2</v>
       </c>
-      <c r="F13" s="87" t="n">
+      <c r="F13" s="83" t="n">
         <v>97.1</v>
       </c>
-      <c r="G13" s="87" t="n">
+      <c r="G13" s="83" t="n">
         <v>110.4</v>
       </c>
-      <c r="H13" s="87" t="n">
+      <c r="H13" s="83" t="n">
         <v>87</v>
       </c>
-      <c r="I13" s="87" t="n">
+      <c r="I13" s="83" t="n">
         <v>91</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="86" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="63" t="s">
         <v>215</v>
       </c>
-      <c r="B14" s="86" t="s">
+      <c r="B14" s="63" t="s">
         <v>239</v>
       </c>
-      <c r="C14" s="87" t="n">
+      <c r="C14" s="83" t="n">
         <v>102.8</v>
       </c>
-      <c r="D14" s="87" t="n">
+      <c r="D14" s="83" t="n">
         <v>117.3</v>
       </c>
-      <c r="E14" s="87" t="n">
+      <c r="E14" s="83" t="n">
         <v>127.8</v>
       </c>
-      <c r="F14" s="87" t="n">
+      <c r="F14" s="83" t="n">
         <v>138</v>
       </c>
-      <c r="G14" s="87" t="n">
+      <c r="G14" s="83" t="n">
         <v>151.6</v>
       </c>
-      <c r="H14" s="87" t="n">
+      <c r="H14" s="83" t="n">
         <v>127.6</v>
       </c>
-      <c r="I14" s="87" t="n">
+      <c r="I14" s="83" t="n">
         <v>134.6</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="86" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="63" t="s">
         <v>438</v>
       </c>
-      <c r="B15" s="86" t="s">
+      <c r="B15" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="87" t="n">
+      <c r="C15" s="83" t="n">
         <v>71.8</v>
       </c>
-      <c r="D15" s="87" t="n">
+      <c r="D15" s="83" t="n">
         <v>78.3</v>
       </c>
-      <c r="E15" s="87" t="n">
+      <c r="E15" s="83" t="n">
         <v>82.9</v>
       </c>
-      <c r="F15" s="87" t="n">
+      <c r="F15" s="83" t="n">
         <v>87.4</v>
       </c>
-      <c r="G15" s="87" t="n">
+      <c r="G15" s="83" t="n">
         <v>93.5</v>
       </c>
-      <c r="H15" s="87" t="n">
+      <c r="H15" s="83" t="n">
         <v>82.8</v>
       </c>
-      <c r="I15" s="87" t="n">
+      <c r="I15" s="83" t="n">
         <v>85</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="86" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="63" t="s">
         <v>438</v>
       </c>
-      <c r="B16" s="86" t="s">
+      <c r="B16" s="63" t="s">
         <v>238</v>
       </c>
-      <c r="C16" s="87" t="n">
+      <c r="C16" s="83" t="n">
         <v>63.2</v>
       </c>
-      <c r="D16" s="87" t="n">
+      <c r="D16" s="83" t="n">
         <v>83.8</v>
       </c>
-      <c r="E16" s="87" t="n">
+      <c r="E16" s="83" t="n">
         <v>98.6</v>
       </c>
-      <c r="F16" s="87" t="n">
+      <c r="F16" s="83" t="n">
         <v>112.9</v>
       </c>
-      <c r="G16" s="87" t="n">
+      <c r="G16" s="83" t="n">
         <v>131.6</v>
       </c>
-      <c r="H16" s="87" t="n">
+      <c r="H16" s="83" t="n">
         <v>98.1</v>
       </c>
-      <c r="I16" s="87" t="n">
+      <c r="I16" s="83" t="n">
         <v>104.3</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="86" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="63" t="s">
         <v>438</v>
       </c>
-      <c r="B17" s="86" t="s">
+      <c r="B17" s="63" t="s">
         <v>239</v>
       </c>
-      <c r="C17" s="87" t="n">
+      <c r="C17" s="83" t="n">
         <v>93</v>
       </c>
-      <c r="D17" s="87" t="n">
+      <c r="D17" s="83" t="n">
         <v>128.2</v>
       </c>
-      <c r="E17" s="87" t="n">
+      <c r="E17" s="83" t="n">
         <v>153.3</v>
       </c>
-      <c r="F17" s="87" t="n">
+      <c r="F17" s="83" t="n">
         <v>177.2</v>
       </c>
-      <c r="G17" s="87" t="n">
+      <c r="G17" s="83" t="n">
         <v>209.8</v>
       </c>
-      <c r="H17" s="87" t="n">
+      <c r="H17" s="83" t="n">
         <v>152.5</v>
       </c>
-      <c r="I17" s="87" t="n">
+      <c r="I17" s="83" t="n">
         <v>165.7</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="84" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="59" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="85" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="58" t="s">
         <v>532</v>
       </c>
-      <c r="B20" s="85"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="85"/>
-      <c r="E20" s="85"/>
-      <c r="F20" s="85"/>
-      <c r="G20" s="85" t="s">
+      <c r="B20" s="58"/>
+      <c r="C20" s="58"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="86" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="63" t="s">
         <v>534</v>
       </c>
-      <c r="G21" s="88" t="n">
+      <c r="G21" s="84" t="n">
         <v>0.898</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="86" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="63" t="s">
         <v>535</v>
       </c>
-      <c r="G22" s="88" t="n">
+      <c r="G22" s="84" t="n">
         <v>0.48</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="86" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="63" t="s">
         <v>536</v>
       </c>
-      <c r="G23" s="88" t="n">
+      <c r="G23" s="84" t="n">
         <v>0.867</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="86" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="63" t="s">
         <v>537</v>
       </c>
-      <c r="G24" s="88" t="n">
+      <c r="G24" s="84" t="n">
         <v>0.01</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="86" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="63" t="s">
         <v>538</v>
       </c>
-      <c r="G25" s="88" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="84" t="s">
+      <c r="G25" s="84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="59" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="85" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="58" t="s">
         <v>322</v>
       </c>
-      <c r="B28" s="85"/>
-      <c r="C28" s="85"/>
-      <c r="D28" s="85" t="s">
+      <c r="B28" s="58"/>
+      <c r="C28" s="58"/>
+      <c r="D28" s="58" t="s">
         <v>540</v>
       </c>
-      <c r="E28" s="85" t="s">
+      <c r="E28" s="58" t="s">
         <v>541</v>
       </c>
-      <c r="F28" s="85" t="s">
+      <c r="F28" s="58" t="s">
         <v>542</v>
       </c>
-      <c r="G28" s="85" t="s">
+      <c r="G28" s="58" t="s">
         <v>543</v>
       </c>
-      <c r="H28" s="85" t="s">
+      <c r="H28" s="58" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="86" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="63" t="s">
         <v>119</v>
       </c>
-      <c r="D29" s="87" t="n">
+      <c r="D29" s="83" t="n">
         <v>191.1</v>
       </c>
-      <c r="E29" s="87" t="n">
+      <c r="E29" s="83" t="n">
         <v>244.2</v>
       </c>
-      <c r="F29" s="87" t="n">
+      <c r="F29" s="83" t="n">
         <v>53</v>
       </c>
-      <c r="G29" s="87" t="n">
+      <c r="G29" s="83" t="n">
         <v>74.9</v>
       </c>
-      <c r="H29" s="87" t="n">
+      <c r="H29" s="83" t="n">
         <v>95.2</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="86" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="63" t="s">
         <v>248</v>
       </c>
-      <c r="D30" s="87" t="n">
+      <c r="D30" s="83" t="n">
         <v>205.2</v>
       </c>
-      <c r="E30" s="87" t="n">
+      <c r="E30" s="83" t="n">
         <v>228</v>
       </c>
-      <c r="F30" s="87" t="n">
+      <c r="F30" s="83" t="n">
         <v>22.8</v>
       </c>
-      <c r="G30" s="87" t="n">
+      <c r="G30" s="83" t="n">
         <v>82.2</v>
       </c>
-      <c r="H30" s="87" t="n">
+      <c r="H30" s="83" t="n">
         <v>87.3</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="86" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="63" t="s">
         <v>428</v>
       </c>
-      <c r="D31" s="87" t="n">
+      <c r="D31" s="83" t="n">
         <v>214.3</v>
       </c>
-      <c r="E31" s="87" t="n">
+      <c r="E31" s="83" t="n">
         <v>221.2</v>
       </c>
-      <c r="F31" s="87" t="n">
+      <c r="F31" s="83" t="n">
         <v>6.9</v>
       </c>
-      <c r="G31" s="87" t="n">
+      <c r="G31" s="83" t="n">
         <v>83.7</v>
       </c>
-      <c r="H31" s="87" t="n">
+      <c r="H31" s="83" t="n">
         <v>86.4</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="86" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="63" t="s">
         <v>332</v>
       </c>
-      <c r="D32" s="87" t="n">
+      <c r="D32" s="83" t="n">
         <v>214.7</v>
       </c>
-      <c r="E32" s="87" t="n">
+      <c r="E32" s="83" t="n">
         <v>220</v>
       </c>
-      <c r="F32" s="87" t="n">
+      <c r="F32" s="83" t="n">
         <v>5.3</v>
       </c>
-      <c r="G32" s="87" t="n">
+      <c r="G32" s="83" t="n">
         <v>84.2</v>
       </c>
-      <c r="H32" s="87" t="n">
+      <c r="H32" s="83" t="n">
         <v>85.3</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="86" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="63" t="s">
         <v>252</v>
       </c>
-      <c r="D33" s="87" t="n">
+      <c r="D33" s="83" t="n">
         <v>214.6</v>
       </c>
-      <c r="E33" s="87" t="n">
+      <c r="E33" s="83" t="n">
         <v>219.6</v>
       </c>
-      <c r="F33" s="87" t="n">
+      <c r="F33" s="83" t="n">
         <v>5</v>
       </c>
-      <c r="G33" s="87" t="n">
+      <c r="G33" s="83" t="n">
         <v>83.7</v>
       </c>
-      <c r="H33" s="87" t="n">
+      <c r="H33" s="83" t="n">
         <v>85.9</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="86" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="63" t="s">
         <v>437</v>
       </c>
-      <c r="D34" s="87" t="n">
+      <c r="D34" s="83" t="n">
         <v>218.5</v>
       </c>
-      <c r="E34" s="87" t="n">
+      <c r="E34" s="83" t="n">
         <v>216.3</v>
       </c>
-      <c r="F34" s="87" t="n">
+      <c r="F34" s="83" t="n">
         <v>-2.2</v>
       </c>
-      <c r="G34" s="87" t="n">
+      <c r="G34" s="83" t="n">
         <v>93.9</v>
       </c>
-      <c r="H34" s="87" t="n">
+      <c r="H34" s="83" t="n">
         <v>61.4</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="86" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="63" t="s">
         <v>545</v>
       </c>
-      <c r="D35" s="87" t="n">
+      <c r="D35" s="83" t="n">
         <v>216.7</v>
       </c>
-      <c r="E35" s="87" t="n">
+      <c r="E35" s="83" t="n">
         <v>218.6</v>
       </c>
-      <c r="F35" s="87" t="n">
+      <c r="F35" s="83" t="n">
         <v>2</v>
       </c>
-      <c r="G35" s="87" t="n">
+      <c r="G35" s="83" t="n">
         <v>84.7</v>
       </c>
-      <c r="H35" s="87" t="n">
+      <c r="H35" s="83" t="n">
         <v>85.4</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="86" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="63" t="s">
         <v>345</v>
       </c>
-      <c r="D36" s="87" t="n">
+      <c r="D36" s="83" t="n">
         <v>217.9</v>
       </c>
-      <c r="E36" s="87" t="n">
+      <c r="E36" s="83" t="n">
         <v>217.4</v>
       </c>
-      <c r="F36" s="87" t="n">
+      <c r="F36" s="83" t="n">
         <v>-0.5</v>
       </c>
-      <c r="G36" s="87" t="n">
+      <c r="G36" s="83" t="n">
         <v>84.6</v>
       </c>
-      <c r="H36" s="87" t="n">
+      <c r="H36" s="83" t="n">
         <v>85.5</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="86" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="63" t="s">
         <v>546</v>
       </c>
-      <c r="D37" s="87" t="n">
+      <c r="D37" s="83" t="n">
         <v>217.7</v>
       </c>
-      <c r="E37" s="87" t="n">
+      <c r="E37" s="83" t="n">
         <v>217.5</v>
       </c>
-      <c r="F37" s="87" t="n">
+      <c r="F37" s="83" t="n">
         <v>-0.1</v>
       </c>
-      <c r="G37" s="87" t="n">
+      <c r="G37" s="83" t="n">
         <v>85.7</v>
       </c>
-      <c r="H37" s="87" t="n">
+      <c r="H37" s="83" t="n">
         <v>83.7</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="84" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="59" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="86" t="s">
+    <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="B40" s="89"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="86" t="s">
+      <c r="B40" s="85" t="s">
+        <v>548</v>
+      </c>
+      <c r="C40" s="85"/>
+      <c r="D40" s="85"/>
+      <c r="E40" s="85"/>
+      <c r="F40" s="85"/>
+      <c r="G40" s="85"/>
+      <c r="H40" s="85"/>
+      <c r="I40" s="85"/>
+    </row>
+    <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="B41" s="89"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="86" t="s">
+      <c r="B41" s="85" t="s">
+        <v>549</v>
+      </c>
+      <c r="C41" s="85"/>
+      <c r="D41" s="85"/>
+      <c r="E41" s="85"/>
+      <c r="F41" s="85"/>
+      <c r="G41" s="85"/>
+      <c r="H41" s="85"/>
+      <c r="I41" s="85"/>
+    </row>
+    <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="63" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="89"/>
+      <c r="B42" s="85" t="s">
+        <v>550</v>
+      </c>
+      <c r="C42" s="85"/>
+      <c r="D42" s="85"/>
+      <c r="E42" s="85"/>
+      <c r="F42" s="85"/>
+      <c r="G42" s="85"/>
+      <c r="H42" s="85"/>
+      <c r="I42" s="85"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B42:I42"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>